<commit_message>
toma de preguntas tests ya estructuradas desde el excel
</commit_message>
<xml_diff>
--- a/backend/preguntas.xlsx
+++ b/backend/preguntas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miguel\OneDrive - UNIVERSIDAD ALICANTE\Escritorio\plataformaopo\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4244169E-694E-4A52-8EBA-6DEEC7A452B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E12AD3-EEC7-421E-B1EE-D8B5E3F60322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{910E72EA-F883-4C38-9DE5-9CDCDBA3BD6B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="21">
   <si>
     <t>tema_id</t>
   </si>
@@ -96,6 +96,9 @@
   </si>
   <si>
     <t>Artículo 1.1 CE: España se constituye en un Estado social y democrático de Derecho, que propugna como valores superiores...</t>
+  </si>
+  <si>
+    <t>numero_test</t>
   </si>
 </sst>
 </file>
@@ -476,10 +479,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39B276DA-A6DA-46D8-8C35-2A497CC075E5}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="55.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.88671875" customWidth="1"/>
     <col min="3" max="3" width="20.6640625" customWidth="1"/>
     <col min="5" max="5" width="21.21875" customWidth="1"/>
     <col min="6" max="6" width="20.6640625" customWidth="1"/>
@@ -487,82 +490,147 @@
     <col min="8" max="8" width="60.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>